<commit_message>
adding cycle time comparision
</commit_message>
<xml_diff>
--- a/results/tables/commitizen/consolidated_results_tables.xlsx
+++ b/results/tables/commitizen/consolidated_results_tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://campusfl-my.sharepoint.com/personal/mahsa_choopannezhad_uni_li/Documents/Desktop/PhD materials/codes/Lifecycles-Processes/results/tables/commitizen/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="11_EB556F4FF53328B727DB86B233B6D209BADD7A48" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12FE7D04-9A34-415F-98D8-EF90CB897BD8}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_EB556F4FF53328B727DB86B233B6D209BADD7A48" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CE08E21-9EFB-496A-B8CF-1C34E312771A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -231,6 +231,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1819,6 +1823,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:P34"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20.453125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>